<commit_message>
Importador: mapeo de columnas nuevas (tipo, tasa IVA/IEPS, stock minimo, tiempo entrega, MOQ, activo)
</commit_message>
<xml_diff>
--- a/ejemplos/plantilla_materias_primas.xlsx
+++ b/ejemplos/plantilla_materias_primas.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\USER\OneDrive\Desktop\AppManufactura\ejemplos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B8B2C42-712B-470F-9027-CC671D4259C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{23629DC6-152E-4977-B159-E9D419298006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A67AFD85-954C-4E9E-84F5-A36E0B7F81DA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{95F5CEF4-0DBA-4DDD-9DA5-31C199AD4A51}"/>
   </bookViews>
   <sheets>
     <sheet name="PLANTILLA" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PLANTILLA!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PLANTILLA!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="64">
   <si>
     <t>Nombre</t>
   </si>
@@ -50,6 +50,9 @@
     <t>SKU</t>
   </si>
   <si>
+    <t>Tipo</t>
+  </si>
+  <si>
     <t>Proveedor</t>
   </si>
   <si>
@@ -62,6 +65,24 @@
     <t>Unidad</t>
   </si>
   <si>
+    <t>Tasa IVA</t>
+  </si>
+  <si>
+    <t>Tasa IEPS</t>
+  </si>
+  <si>
+    <t>Stock minimo</t>
+  </si>
+  <si>
+    <t>Tiempo entrega dias</t>
+  </si>
+  <si>
+    <t>Cantidad minima compra</t>
+  </si>
+  <si>
+    <t>Activo</t>
+  </si>
+  <si>
     <t>Notas</t>
   </si>
   <si>
@@ -71,6 +92,9 @@
     <t>MP-CMC</t>
   </si>
   <si>
+    <t>materia prima</t>
+  </si>
+  <si>
     <t>ALKEM</t>
   </si>
   <si>
@@ -80,6 +104,9 @@
     <t>Kilogramos</t>
   </si>
   <si>
+    <t>si</t>
+  </si>
+  <si>
     <t>Carboximetilcelulosa - espesante</t>
   </si>
   <si>
@@ -183,6 +210,9 @@
   </si>
   <si>
     <t>INS-ENVASE-PET-60</t>
+  </si>
+  <si>
+    <t>insumo</t>
   </si>
   <si>
     <t>ESCOWILL</t>
@@ -253,8 +283,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -589,320 +620,590 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC3B639D-4093-4A9D-BFFA-8883D69065A9}">
-  <dimension ref="A1:G13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B254E14A-0764-402A-8576-F67F1E0B0C34}">
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="14" max="14" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2">
+        <v>180</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>25</v>
+      </c>
+      <c r="K2">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2">
-        <v>180</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="L2">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <v>60</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>50</v>
+      </c>
+      <c r="K3">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
+      <c r="L3">
+        <v>200</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
+      </c>
+      <c r="N3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>50</v>
+      </c>
+      <c r="K4">
+        <v>10</v>
+      </c>
+      <c r="L4">
+        <v>200</v>
+      </c>
+      <c r="M4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5">
+        <v>160</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>10</v>
+      </c>
+      <c r="K5">
+        <v>7</v>
+      </c>
+      <c r="L5">
+        <v>25</v>
+      </c>
+      <c r="M5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6">
+        <v>90</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6">
+        <v>7</v>
+      </c>
+      <c r="L6">
+        <v>25</v>
+      </c>
+      <c r="M6" t="s">
+        <v>20</v>
+      </c>
+      <c r="N6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>100</v>
+      </c>
+      <c r="K7">
+        <v>3</v>
+      </c>
+      <c r="L7">
+        <v>200</v>
+      </c>
+      <c r="M7" t="s">
+        <v>20</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8">
+        <v>240</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>20</v>
+      </c>
+      <c r="K8">
+        <v>15</v>
+      </c>
+      <c r="L8">
+        <v>20</v>
+      </c>
+      <c r="M8" t="s">
+        <v>20</v>
+      </c>
+      <c r="N8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9">
+        <v>39</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>10</v>
+      </c>
+      <c r="L9">
+        <v>200</v>
+      </c>
+      <c r="M9" t="s">
+        <v>20</v>
+      </c>
+      <c r="N9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10">
+        <v>550</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+      <c r="K10">
+        <v>20</v>
+      </c>
+      <c r="L10">
+        <v>5</v>
+      </c>
+      <c r="M10" t="s">
+        <v>20</v>
+      </c>
+      <c r="N10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11">
+        <v>780</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+      <c r="K11">
+        <v>30</v>
+      </c>
+      <c r="L11">
+        <v>10</v>
+      </c>
+      <c r="M11" t="s">
+        <v>20</v>
+      </c>
+      <c r="N11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12">
+        <v>3.1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>500</v>
+      </c>
+      <c r="K12">
+        <v>20</v>
+      </c>
+      <c r="L12">
+        <v>1000</v>
+      </c>
+      <c r="M12" t="s">
+        <v>20</v>
+      </c>
+      <c r="N12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>60</v>
       </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13">
+        <v>1.85</v>
+      </c>
+      <c r="F13" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4">
-        <v>50</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5">
-        <v>160</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>90</v>
-      </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8">
-        <v>240</v>
-      </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9">
-        <v>39</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10">
-        <v>550</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11">
-        <v>780</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12">
-        <v>3.1</v>
-      </c>
-      <c r="E12" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" t="s">
-        <v>48</v>
-      </c>
-      <c r="G12" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13">
-        <v>1.85</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>48</v>
-      </c>
       <c r="G13" t="s">
-        <v>53</v>
+        <v>58</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>500</v>
+      </c>
+      <c r="K13">
+        <v>20</v>
+      </c>
+      <c r="L13">
+        <v>1000</v>
+      </c>
+      <c r="M13" t="s">
+        <v>20</v>
+      </c>
+      <c r="N13" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{DC3B639D-4093-4A9D-BFFA-8883D69065A9}"/>
+  <autoFilter ref="A1:N1" xr:uid="{B254E14A-0764-402A-8576-F67F1E0B0C34}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Precio de venta por producto: catalogo + CSV + calculo automatico en ventas + contabilizar ventas viejas desde el historial
</commit_message>
<xml_diff>
--- a/ejemplos/plantilla_materias_primas.xlsx
+++ b/ejemplos/plantilla_materias_primas.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\USER\OneDrive\Desktop\AppManufactura\ejemplos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23629DC6-152E-4977-B159-E9D419298006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{729AFCF2-4685-414F-9D67-E1E3B08FC145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{95F5CEF4-0DBA-4DDD-9DA5-31C199AD4A51}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B41ECBC-E95E-4380-BB29-EDD9AA1B571A}"/>
   </bookViews>
   <sheets>
     <sheet name="PLANTILLA" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PLANTILLA!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PLANTILLA!$A$1:$O$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="69">
   <si>
     <t>Nombre</t>
   </si>
@@ -59,6 +59,9 @@
     <t>Precio</t>
   </si>
   <si>
+    <t>Precio de venta</t>
+  </si>
+  <si>
     <t>Moneda</t>
   </si>
   <si>
@@ -206,6 +209,21 @@
     <t>Saborizante chicle</t>
   </si>
   <si>
+    <t>Gel lubricante 60 ml</t>
+  </si>
+  <si>
+    <t>PT-GEL-60</t>
+  </si>
+  <si>
+    <t>producto</t>
+  </si>
+  <si>
+    <t>Piezas</t>
+  </si>
+  <si>
+    <t>Producto terminado - ejemplo con precio de venta</t>
+  </si>
+  <si>
     <t>Envase PET 60 ml</t>
   </si>
   <si>
@@ -216,9 +234,6 @@
   </si>
   <si>
     <t>ESCOWILL</t>
-  </si>
-  <si>
-    <t>Piezas</t>
   </si>
   <si>
     <t>Envase tipo Boston 60 ml</t>
@@ -620,17 +635,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B254E14A-0764-402A-8576-F67F1E0B0C34}">
-  <dimension ref="A1:N13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53CD1343-AC7D-45F4-A0EF-3A9D35311A6E}">
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
     <col min="4" max="4" width="22.7109375" customWidth="1"/>
-    <col min="14" max="14" width="30.7109375" customWidth="1"/>
+    <col min="15" max="15" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -673,492 +688,495 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2">
         <v>180</v>
       </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
       <c r="G2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="1">
         <v>0.16</v>
       </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
         <v>25</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>7</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>25</v>
-      </c>
-      <c r="M2" t="s">
-        <v>20</v>
       </c>
       <c r="N2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3">
         <v>60</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>50</v>
+      </c>
+      <c r="L3">
+        <v>10</v>
+      </c>
+      <c r="M3">
+        <v>200</v>
+      </c>
+      <c r="N3" t="s">
+        <v>21</v>
+      </c>
+      <c r="O3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
         <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="1">
-        <v>0.16</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>50</v>
-      </c>
-      <c r="K3">
-        <v>10</v>
-      </c>
-      <c r="L3">
-        <v>200</v>
-      </c>
-      <c r="M3" t="s">
-        <v>20</v>
-      </c>
-      <c r="N3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
       </c>
       <c r="E4">
         <v>50</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>50</v>
+      </c>
+      <c r="L4">
+        <v>10</v>
+      </c>
+      <c r="M4">
+        <v>200</v>
+      </c>
+      <c r="N4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
         <v>18</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0.16</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>50</v>
-      </c>
-      <c r="K4">
-        <v>10</v>
-      </c>
-      <c r="L4">
-        <v>200</v>
-      </c>
-      <c r="M4" t="s">
-        <v>20</v>
-      </c>
-      <c r="N4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
       </c>
       <c r="E5">
         <v>160</v>
       </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
       <c r="G5" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="1">
         <v>0.16</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
       <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
         <v>10</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>7</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>25</v>
       </c>
-      <c r="M5" t="s">
-        <v>20</v>
-      </c>
       <c r="N5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="O5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>90</v>
       </c>
-      <c r="F6" t="s">
-        <v>18</v>
-      </c>
       <c r="G6" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="1">
         <v>0.16</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
       <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
         <v>5</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>7</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>25</v>
       </c>
-      <c r="M6" t="s">
-        <v>20</v>
-      </c>
       <c r="N6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="O6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
-      <c r="F7" t="s">
-        <v>18</v>
-      </c>
       <c r="G7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0</v>
-      </c>
-      <c r="I7">
+        <v>19</v>
+      </c>
+      <c r="H7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="1">
         <v>0</v>
       </c>
       <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
         <v>100</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>3</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>200</v>
       </c>
-      <c r="M7" t="s">
-        <v>20</v>
-      </c>
       <c r="N7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="O7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E8">
         <v>240</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>20</v>
+      </c>
+      <c r="L8">
+        <v>15</v>
+      </c>
+      <c r="M8">
+        <v>20</v>
+      </c>
+      <c r="N8" t="s">
+        <v>21</v>
+      </c>
+      <c r="O8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
         <v>18</v>
-      </c>
-      <c r="G8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H8" s="1">
-        <v>0.16</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>20</v>
-      </c>
-      <c r="K8">
-        <v>15</v>
-      </c>
-      <c r="L8">
-        <v>20</v>
-      </c>
-      <c r="M8" t="s">
-        <v>20</v>
-      </c>
-      <c r="N8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>17</v>
       </c>
       <c r="E9">
         <v>39</v>
       </c>
-      <c r="F9" t="s">
-        <v>18</v>
-      </c>
       <c r="G9" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" s="1">
+        <v>19</v>
+      </c>
+      <c r="H9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="1">
         <v>0.16</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
       <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
         <v>20</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>10</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>200</v>
       </c>
-      <c r="M9" t="s">
-        <v>20</v>
-      </c>
       <c r="N9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="O9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E10">
         <v>550</v>
       </c>
-      <c r="F10" t="s">
-        <v>18</v>
-      </c>
       <c r="G10" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="1">
         <v>0.16</v>
       </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
       <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
         <v>2</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>20</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>5</v>
       </c>
-      <c r="M10" t="s">
-        <v>20</v>
-      </c>
       <c r="N10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="O10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E11">
         <v>780</v>
       </c>
-      <c r="F11" t="s">
-        <v>18</v>
-      </c>
       <c r="G11" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" s="1">
+        <v>19</v>
+      </c>
+      <c r="H11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" s="1">
         <v>0.16</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
       <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
         <v>3</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>30</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>10</v>
       </c>
-      <c r="M11" t="s">
-        <v>20</v>
-      </c>
       <c r="N11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="O11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" t="s">
         <v>57</v>
       </c>
       <c r="E12">
-        <v>3.1</v>
-      </c>
-      <c r="F12" t="s">
-        <v>18</v>
+        <v>18.5</v>
+      </c>
+      <c r="F12">
+        <v>45</v>
       </c>
       <c r="G12" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" t="s">
         <v>58</v>
       </c>
-      <c r="H12" s="1">
+      <c r="I12" s="1">
         <v>0.16</v>
       </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
       <c r="J12">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="L12">
-        <v>1000</v>
-      </c>
-      <c r="M12" t="s">
-        <v>20</v>
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
       </c>
       <c r="N12" t="s">
+        <v>21</v>
+      </c>
+      <c r="O12" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>60</v>
       </c>
@@ -1166,44 +1184,88 @@
         <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13">
+        <v>3.1</v>
+      </c>
+      <c r="G13" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" t="s">
+        <v>58</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>500</v>
+      </c>
+      <c r="L13">
+        <v>20</v>
+      </c>
+      <c r="M13">
+        <v>1000</v>
+      </c>
+      <c r="N13" t="s">
+        <v>21</v>
+      </c>
+      <c r="O13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" t="s">
         <v>62</v>
       </c>
-      <c r="E13">
+      <c r="D14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14">
         <v>1.85</v>
       </c>
-      <c r="F13" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="G14" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" t="s">
         <v>58</v>
       </c>
-      <c r="H13" s="1">
+      <c r="I14" s="1">
         <v>0.16</v>
       </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
         <v>500</v>
       </c>
-      <c r="K13">
+      <c r="L14">
         <v>20</v>
       </c>
-      <c r="L13">
+      <c r="M14">
         <v>1000</v>
       </c>
-      <c r="M13" t="s">
-        <v>20</v>
-      </c>
-      <c r="N13" t="s">
-        <v>63</v>
+      <c r="N14" t="s">
+        <v>21</v>
+      </c>
+      <c r="O14" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{B254E14A-0764-402A-8576-F67F1E0B0C34}"/>
+  <autoFilter ref="A1:O1" xr:uid="{53CD1343-AC7D-45F4-A0EF-3A9D35311A6E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>